<commit_message>
Weekly refresh of the Denver crash extracts
</commit_message>
<xml_diff>
--- a/reports/two_death_counts.xlsx
+++ b/reports/two_death_counts.xlsx
@@ -854,7 +854,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>17905</v>
+        <v>17904</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>41</v>
@@ -889,16 +889,16 @@
         <v>1</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>14578</v>
+        <v>14838</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>26</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>0</v>
@@ -907,7 +907,7 @@
         <v>5</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>0</v>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Pedestrian-involved crashes in the file: 2021: 404, 2022: 374, 2023: 522, 2024: 494, 2025: 463, 2026: 357. Pedestrian deaths in that file (FATALITIES on pedestrian_ind rows, and fatality mode): 2021: 15, 2022: 3, 2023: 0, 2024: 0, 2025: 0, 2026: 0. Fatality-mode pedestrian deaths in 2025: 0. DOTI, via the Gazette: 35 pedestrian deaths in 2025.</t>
+          <t>Pedestrian-involved crashes in the file: 2021: 404, 2022: 374, 2023: 522, 2024: 494, 2025: 463, 2026: 360. Pedestrian deaths in that file (FATALITIES on pedestrian_ind rows, and fatality mode): 2021: 15, 2022: 3, 2023: 0, 2024: 0, 2025: 0, 2026: 0. Fatality-mode pedestrian deaths in 2025: 0. DOTI, via the Gazette: 35 pedestrian deaths in 2025.</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -1486,7 +1486,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>COLORADO BLVD</t>
+          <t>ALAMEDA AVE</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -1496,7 +1496,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>ALAMEDA AVE</t>
+          <t>COLORADO BLVD</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -1536,7 +1536,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>PARK AVEW</t>
+          <t>SPEER BLVD</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
@@ -1546,7 +1546,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>SPEER BLVD</t>
+          <t>PARK AVEW</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -1576,7 +1576,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>8TH AVE</t>
+          <t>MISSISSIPPI AVE</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
@@ -1586,7 +1586,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>11TH AVE</t>
+          <t>8TH AVE</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">

</xml_diff>